<commit_message>
Billions: que no se repitan las mismas películas
Son 100 películas, pero dos cosas hacían que parecieran muchas menos.

Nada impedía preguntar dos veces por la misma película en una partida:
en 20 rondas se repetía alguna el 99 % de las veces, 3,8 de media. Ahora
se lleva registro de las ya preguntadas y los generadores trabajan sobre
el depósito filtrado; si quedasen menos de diez sin usar se vuelve al
depósito entero, antes que quedarse sin preguntas.

Y los depósitos de imagen de fondo de las burbujas eran diminutos: 18
carátulas de taquilla, 13 de estrenos y 16 premiadas, con cuatro
burbujas de cada categoría por partida. Pasan a 45, 32 y 27.

Repeticiones por partida: 3,8 -> 0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/top_peliculas_taquilla_y_critica.xlsx
+++ b/top_peliculas_taquilla_y_critica.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,15 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00666666"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00CCCCCC"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -145,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -203,6 +212,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -568,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -583,6 +604,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="65" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -660,6 +682,11 @@
           <t>Actor 5</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Categorías de Oscar</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -712,6 +739,11 @@
           <t>Michelle Rodriguez</t>
         </is>
       </c>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejores Efectos Visuales, Mejor Dirección Artística</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -764,6 +796,11 @@
           <t>Chris Hemsworth</t>
         </is>
       </c>
+      <c r="M6" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -816,6 +853,11 @@
           <t>Stephen Lang</t>
         </is>
       </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -868,6 +910,11 @@
           <t>Frances Fisher</t>
         </is>
       </c>
+      <c r="M8" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido, Mejor Banda Sonora, Mejor Canción Original, Mejor Fotografía, Mejor Dirección Artística, Mejor Vestuario, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -920,6 +967,11 @@
           <t>Oscar Isaac</t>
         </is>
       </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -972,6 +1024,11 @@
           <t>Scarlett Johansson</t>
         </is>
       </c>
+      <c r="M10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1026,6 +1083,11 @@
           <t>Jon Favreau</t>
         </is>
       </c>
+      <c r="M11" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -1080,6 +1142,11 @@
           <t>Liu Tongzi</t>
         </is>
       </c>
+      <c r="M12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1132,6 +1199,11 @@
           <t>Andrew Garfield</t>
         </is>
       </c>
+      <c r="M13" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -1186,6 +1258,11 @@
           <t>Idris Elba</t>
         </is>
       </c>
+      <c r="M14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1238,6 +1315,11 @@
           <t>Phyllis Smith</t>
         </is>
       </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -1290,6 +1372,11 @@
           <t>Nick Robinson</t>
         </is>
       </c>
+      <c r="M16" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1342,6 +1429,11 @@
           <t>Chiwetel Ejiofor</t>
         </is>
       </c>
+      <c r="M17" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -1394,6 +1486,11 @@
           <t>Chris Hemsworth</t>
         </is>
       </c>
+      <c r="M18" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1446,6 +1543,11 @@
           <t>Michelle Rodriguez</t>
         </is>
       </c>
+      <c r="M19" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -1500,6 +1602,11 @@
           <t>Oona Chaplin</t>
         </is>
       </c>
+      <c r="M20" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1552,6 +1659,11 @@
           <t>Glen Powell</t>
         </is>
       </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -1604,6 +1716,11 @@
           <t>Sterling K. Brown</t>
         </is>
       </c>
+      <c r="M22" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1656,6 +1773,11 @@
           <t>America Ferrera</t>
         </is>
       </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -1708,6 +1830,11 @@
           <t>Scarlett Johansson</t>
         </is>
       </c>
+      <c r="M24" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -1760,6 +1887,11 @@
           <t>Keegan-Michael Key</t>
         </is>
       </c>
+      <c r="M25" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -1814,6 +1946,11 @@
           <t>Charlize Theron</t>
         </is>
       </c>
+      <c r="M26" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1866,6 +2003,11 @@
           <t>Matthew Macfadyen</t>
         </is>
       </c>
+      <c r="M27" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -1918,6 +2060,11 @@
           <t>Letitia Wright</t>
         </is>
       </c>
+      <c r="M28" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario, Mejor Diseño de Producción, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1970,6 +2117,11 @@
           <t>John Boyega</t>
         </is>
       </c>
+      <c r="M29" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -2022,6 +2174,11 @@
           <t>Alan Rickman</t>
         </is>
       </c>
+      <c r="M30" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -2074,6 +2231,11 @@
           <t>James Cromwell</t>
         </is>
       </c>
+      <c r="M31" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -2126,6 +2288,11 @@
           <t>Santino Fontana</t>
         </is>
       </c>
+      <c r="M32" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -2178,6 +2345,11 @@
           <t>Josh Gad</t>
         </is>
       </c>
+      <c r="M33" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
@@ -2230,6 +2402,11 @@
           <t>Huck Milner</t>
         </is>
       </c>
+      <c r="M34" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -2282,6 +2459,11 @@
           <t>Ben Kingsley</t>
         </is>
       </c>
+      <c r="M35" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
@@ -2334,6 +2516,11 @@
           <t>Michelle Rodriguez</t>
         </is>
       </c>
+      <c r="M36" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -2386,6 +2573,11 @@
           <t>Pierre Coffin</t>
         </is>
       </c>
+      <c r="M37" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -2438,6 +2630,11 @@
           <t>Chadwick Boseman</t>
         </is>
       </c>
+      <c r="M38" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -2490,6 +2687,11 @@
           <t>Nicole Kidman</t>
         </is>
       </c>
+      <c r="M39" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -2542,6 +2744,11 @@
           <t>Marisa Tomei</t>
         </is>
       </c>
+      <c r="M40" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -2594,6 +2801,11 @@
           <t>Annette Bening</t>
         </is>
       </c>
+      <c r="M41" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -2646,6 +2858,11 @@
           <t>Orlando Bloom</t>
         </is>
       </c>
+      <c r="M42" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Maquillaje, Mejor Banda Sonora, Mejor Canción Original, Mejor Mezcla de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -2698,6 +2915,11 @@
           <t>Tyrese Gibson</t>
         </is>
       </c>
+      <c r="M43" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
@@ -2752,6 +2974,11 @@
           <t>Joan Cusack</t>
         </is>
       </c>
+      <c r="M44" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2804,6 +3031,11 @@
           <t>Naomie Harris</t>
         </is>
       </c>
+      <c r="M45" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n">
@@ -2856,6 +3088,11 @@
           <t>Jack Reynor</t>
         </is>
       </c>
+      <c r="M46" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2908,6 +3145,11 @@
           <t>Gary Oldman</t>
         </is>
       </c>
+      <c r="M47" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
@@ -2960,6 +3202,11 @@
           <t>Brett Cullen</t>
         </is>
       </c>
+      <c r="M48" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -3012,6 +3259,11 @@
           <t>Keegan-Michael Key</t>
         </is>
       </c>
+      <c r="M49" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n">
@@ -3064,6 +3316,11 @@
           <t>Mark Hamill</t>
         </is>
       </c>
+      <c r="M50" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -3116,6 +3373,11 @@
           <t>Michael Keaton</t>
         </is>
       </c>
+      <c r="M51" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
@@ -3168,6 +3430,11 @@
           <t>Stellan Skarsgård</t>
         </is>
       </c>
+      <c r="M52" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -3220,6 +3487,11 @@
           <t>David Fane</t>
         </is>
       </c>
+      <c r="M53" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
@@ -3272,6 +3544,11 @@
           <t>Samuel L. Jackson</t>
         </is>
       </c>
+      <c r="M54" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -3324,6 +3601,11 @@
           <t>Ben Mendelsohn</t>
         </is>
       </c>
+      <c r="M55" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n">
@@ -3376,6 +3658,11 @@
           <t>Ian McDiarmid</t>
         </is>
       </c>
+      <c r="M56" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -3428,6 +3715,11 @@
           <t>Kevin McNally</t>
         </is>
       </c>
+      <c r="M57" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n">
@@ -3480,6 +3772,11 @@
           <t>Navid Negahban</t>
         </is>
       </c>
+      <c r="M58" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -3534,6 +3831,11 @@
           <t>Billy Magnussen</t>
         </is>
       </c>
+      <c r="M59" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n">
@@ -3586,6 +3888,11 @@
           <t>Miranda Cosgrove</t>
         </is>
       </c>
+      <c r="M60" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -3638,6 +3945,11 @@
           <t>Crispin Glover</t>
         </is>
       </c>
+      <c r="M61" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Dirección Artística, Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n">
@@ -3690,6 +4002,11 @@
           <t>Ty Burrell</t>
         </is>
       </c>
+      <c r="M62" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -3742,6 +4059,11 @@
           <t>Nate Torrence</t>
         </is>
       </c>
+      <c r="M63" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n">
@@ -3794,6 +4116,11 @@
           <t>Hugo Weaving</t>
         </is>
       </c>
+      <c r="M64" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -3846,6 +4173,11 @@
           <t>Gary Oldman</t>
         </is>
       </c>
+      <c r="M65" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Heath Ledger), Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n">
@@ -3898,6 +4230,11 @@
           <t>Jeff Goldblum</t>
         </is>
       </c>
+      <c r="M66" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -3950,6 +4287,11 @@
           <t>Ernie Sabella</t>
         </is>
       </c>
+      <c r="M67" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Banda Sonora, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n">
@@ -4002,6 +4344,11 @@
           <t>Joey King</t>
         </is>
       </c>
+      <c r="M68" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -4054,6 +4401,11 @@
           <t>Florence Pugh</t>
         </is>
       </c>
+      <c r="M69" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actor de Reparto, Mejor Montaje, Mejor Fotografía, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n">
@@ -4106,6 +4458,11 @@
           <t>Russell Brand</t>
         </is>
       </c>
+      <c r="M70" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -4158,6 +4515,11 @@
           <t>Maggie Smith</t>
         </is>
       </c>
+      <c r="M71" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n">
@@ -4210,6 +4572,11 @@
           <t>Nick Jonas</t>
         </is>
       </c>
+      <c r="M72" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -4264,6 +4631,11 @@
           <t>Jennifer Coolidge</t>
         </is>
       </c>
+      <c r="M73" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n">
@@ -4316,6 +4688,11 @@
           <t>Bill Nighy</t>
         </is>
       </c>
+      <c r="M74" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -4368,6 +4745,11 @@
           <t>Orlando Bloom</t>
         </is>
       </c>
+      <c r="M75" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n">
@@ -4420,6 +4802,11 @@
           <t>Chiwetel Ejiofor</t>
         </is>
       </c>
+      <c r="M76" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -4472,6 +4859,11 @@
           <t>Scarlett Johansson</t>
         </is>
       </c>
+      <c r="M77" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n">
@@ -4524,6 +4916,11 @@
           <t>Alan Rickman</t>
         </is>
       </c>
+      <c r="M78" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -4576,6 +4973,11 @@
           <t>Benedict Cumberbatch</t>
         </is>
       </c>
+      <c r="M79" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n">
@@ -4628,6 +5030,11 @@
           <t>Jean-Claude Van Damme</t>
         </is>
       </c>
+      <c r="M80" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -4680,6 +5087,11 @@
           <t>Ralph Fiennes</t>
         </is>
       </c>
+      <c r="M81" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n">
@@ -4732,6 +5144,11 @@
           <t>Geoffrey Rush</t>
         </is>
       </c>
+      <c r="M82" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -4784,6 +5201,11 @@
           <t>Julie Andrews</t>
         </is>
       </c>
+      <c r="M83" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n">
@@ -4836,6 +5258,11 @@
           <t>Sean Astin</t>
         </is>
       </c>
+      <c r="M84" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4888,6 +5315,11 @@
           <t>Alan Rickman</t>
         </is>
       </c>
+      <c r="M85" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n">
@@ -4940,6 +5372,11 @@
           <t>Samuel L. Jackson</t>
         </is>
       </c>
+      <c r="M86" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -4992,6 +5429,11 @@
           <t>Orlando Bloom</t>
         </is>
       </c>
+      <c r="M87" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Maquillaje, Mejor Banda Sonora, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n">
@@ -5044,6 +5486,11 @@
           <t>Topher Grace</t>
         </is>
       </c>
+      <c r="M88" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -5096,6 +5543,11 @@
           <t>Robert Pattinson</t>
         </is>
       </c>
+      <c r="M89" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n">
@@ -5148,6 +5600,11 @@
           <t>Simon Pegg</t>
         </is>
       </c>
+      <c r="M90" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -5200,6 +5657,11 @@
           <t>Ellie Kemper</t>
         </is>
       </c>
+      <c r="M91" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n">
@@ -5252,6 +5714,11 @@
           <t>Jennifer Lopez</t>
         </is>
       </c>
+      <c r="M92" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -5304,6 +5771,11 @@
           <t>Joseph Mazzello</t>
         </is>
       </c>
+      <c r="M93" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Montaje, Mejor Edición de Sonido, Mejor Mezcla de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n">
@@ -5356,6 +5828,11 @@
           <t>Monica Bellucci</t>
         </is>
       </c>
+      <c r="M94" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -5408,6 +5885,11 @@
           <t>Marisa Tomei</t>
         </is>
       </c>
+      <c r="M95" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n">
@@ -5460,6 +5942,11 @@
           <t>Alan Rickman</t>
         </is>
       </c>
+      <c r="M96" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
@@ -5512,6 +5999,11 @@
           <t>Gal Gadot</t>
         </is>
       </c>
+      <c r="M97" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n">
@@ -5566,6 +6058,11 @@
           <t>Manuel Garcia-Rulfo</t>
         </is>
       </c>
+      <c r="M98" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -5618,6 +6115,11 @@
           <t>Bradley Cooper</t>
         </is>
       </c>
+      <c r="M99" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n">
@@ -5670,6 +6172,11 @@
           <t>Woody Harrelson</t>
         </is>
       </c>
+      <c r="M100" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
@@ -5722,6 +6229,11 @@
           <t>Tenoch Huerta</t>
         </is>
       </c>
+      <c r="M101" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n">
@@ -5774,7 +6286,13 @@
           <t>Jenny Slate</t>
         </is>
       </c>
-    </row>
+      <c r="M102" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="103"/>
     <row r="104">
       <c r="A104" s="18" t="inlineStr">
         <is>
@@ -5799,7 +6317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5814,6 +6332,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="65" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5891,6 +6410,11 @@
           <t>Actor 5</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Categorías de Oscar</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -5943,6 +6467,11 @@
           <t>Diane Keaton</t>
         </is>
       </c>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -5995,6 +6524,11 @@
           <t>John Cazale</t>
         </is>
       </c>
+      <c r="M6" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion Adaptado, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -6047,6 +6581,11 @@
           <t>Ed Begley</t>
         </is>
       </c>
+      <c r="M7" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -6099,6 +6638,11 @@
           <t>Embeth Davidtz</t>
         </is>
       </c>
+      <c r="M8" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje, Mejor Fotografía, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -6151,6 +6695,11 @@
           <t>Tim Roth</t>
         </is>
       </c>
+      <c r="M9" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -6203,6 +6752,11 @@
           <t>Clancy Brown</t>
         </is>
       </c>
+      <c r="M10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -6255,6 +6809,11 @@
           <t>Al Ernest Garcia</t>
         </is>
       </c>
+      <c r="M11" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -6307,6 +6866,11 @@
           <t>Henry Daniell</t>
         </is>
       </c>
+      <c r="M12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -6359,6 +6923,11 @@
           <t>Chester Conklin</t>
         </is>
       </c>
+      <c r="M13" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -6413,6 +6982,11 @@
           <t>John Williams</t>
         </is>
       </c>
+      <c r="M14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -6465,6 +7039,11 @@
           <t>Ray Walston</t>
         </is>
       </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -6517,6 +7096,11 @@
           <t>Horst Buchholz</t>
         </is>
       </c>
+      <c r="M16" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Película de Habla No Inglesa, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -6569,6 +7153,11 @@
           <t>Fred Clark</t>
         </is>
       </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Guion, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -6623,6 +7212,11 @@
           <t>Lionel Atwill</t>
         </is>
       </c>
+      <c r="M18" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -6677,6 +7271,11 @@
           <t>Gary Merrill</t>
         </is>
       </c>
+      <c r="M19" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion, Mejor Vestuario, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -6729,6 +7328,11 @@
           <t>Jack Kruschen</t>
         </is>
       </c>
+      <c r="M20" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Dirección Artística, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -6781,6 +7385,11 @@
           <t>Conrad Veidt</t>
         </is>
       </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -6833,6 +7442,11 @@
           <t>Paul Sorvino</t>
         </is>
       </c>
+      <c r="M22" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Joe Pesci)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -6885,6 +7499,11 @@
           <t>Martin Balsam</t>
         </is>
       </c>
+      <c r="M23" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -6937,6 +7556,11 @@
           <t>Jonathan Haagensen</t>
         </is>
       </c>
+      <c r="M24" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -6989,6 +7613,11 @@
           <t>Isao Kimura</t>
         </is>
       </c>
+      <c r="M25" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -7043,6 +7672,11 @@
           <t>Wayne Morris</t>
         </is>
       </c>
+      <c r="M26" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -7095,6 +7729,11 @@
           <t>Raymond Burr</t>
         </is>
       </c>
+      <c r="M27" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -7147,6 +7786,11 @@
           <t>Mykelti Williamson</t>
         </is>
       </c>
+      <c r="M28" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Montaje, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -7199,6 +7843,11 @@
           <t>Alec Guinness</t>
         </is>
       </c>
+      <c r="M29" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Sonido, Premio Especial Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -7251,6 +7900,11 @@
           <t>Agnes Moorehead</t>
         </is>
       </c>
+      <c r="M30" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -7303,6 +7957,11 @@
           <t>Yasuko Sawaguchi</t>
         </is>
       </c>
+      <c r="M31" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -7355,6 +8014,11 @@
           <t>Agnese Nano</t>
         </is>
       </c>
+      <c r="M32" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Habla No Inglesa</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -7409,6 +8073,11 @@
           <t>Minoru Chiaki</t>
         </is>
       </c>
+      <c r="M33" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Habla No Inglesa (Premio Honorífico)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
@@ -7461,6 +8130,11 @@
           <t>Henry Jones</t>
         </is>
       </c>
+      <c r="M34" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -7513,6 +8187,11 @@
           <t>Millard Mitchell</t>
         </is>
       </c>
+      <c r="M35" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
@@ -7565,6 +8244,11 @@
           <t>Gabriele Ferzetti</t>
         </is>
       </c>
+      <c r="M36" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -7617,6 +8301,11 @@
           <t>Roy Dotrice</t>
         </is>
       </c>
+      <c r="M37" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Dirección Artística, Mejor Vestuario, Mejor Maquillaje, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -7669,6 +8358,11 @@
           <t>José Ferrer</t>
         </is>
       </c>
+      <c r="M38" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Fotografía, Mejor Dirección Artística, Mejor Montaje, Mejor Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -7721,6 +8415,11 @@
           <t>Anthony Heald</t>
         </is>
       </c>
+      <c r="M39" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actriz, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -7773,6 +8472,11 @@
           <t>Christopher Lloyd</t>
         </is>
       </c>
+      <c r="M40" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actriz, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -7825,6 +8529,11 @@
           <t>Park So-dam</t>
         </is>
       </c>
+      <c r="M41" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Película Internacional</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -7877,6 +8586,11 @@
           <t>Maureen Lipman</t>
         </is>
       </c>
+      <c r="M42" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actor, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -7929,6 +8643,11 @@
           <t>Frank Vincent</t>
         </is>
       </c>
+      <c r="M43" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
@@ -7981,6 +8700,11 @@
           <t>Leonard Rossiter</t>
         </is>
       </c>
+      <c r="M44" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -8033,6 +8757,11 @@
           <t>George Raft</t>
         </is>
       </c>
+      <c r="M45" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n">
@@ -8085,6 +8814,11 @@
           <t>Jared Leto</t>
         </is>
       </c>
+      <c r="M46" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -8137,6 +8871,11 @@
           <t>Luigi Pistilli</t>
         </is>
       </c>
+      <c r="M47" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
@@ -8189,6 +8928,11 @@
           <t>James Donald</t>
         </is>
       </c>
+      <c r="M48" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Fotografía, Mejor Montaje, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -8241,6 +8985,11 @@
           <t>Peter Cushing</t>
         </is>
       </c>
+      <c r="M49" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Sonido, Mejores Efectos Visuales, Mejor Banda Sonora, Premio Especial Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n">
@@ -8293,6 +9042,11 @@
           <t>Barry Pepper</t>
         </is>
       </c>
+      <c r="M50" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Fotografía, Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -8345,6 +9099,11 @@
           <t>Ken Watanabe</t>
         </is>
       </c>
+      <c r="M51" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Mezcla de Sonido, Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
@@ -8397,6 +9156,11 @@
           <t>Joe Morton</t>
         </is>
       </c>
+      <c r="M52" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido, Mejor Maquillaje</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -8449,6 +9213,11 @@
           <t>Austin Stowell</t>
         </is>
       </c>
+      <c r="M53" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Montaje, Mejor Mezcla de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
@@ -8501,6 +9270,11 @@
           <t>Stephen Baldwin</t>
         </is>
       </c>
+      <c r="M54" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -8553,6 +9327,11 @@
           <t>Laurence Fishburne</t>
         </is>
       </c>
+      <c r="M55" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n">
@@ -8605,6 +9384,11 @@
           <t>James Cromwell</t>
         </is>
       </c>
+      <c r="M56" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -8657,6 +9441,11 @@
           <t>Martha Scott</t>
         </is>
       </c>
+      <c r="M57" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actor de Reparto, Mejor Fotografía, Mejor Dirección Artística, Mejor Vestuario, Mejor Montaje, Mejor Sonido, Mejores Efectos Visuales, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n">
@@ -8709,6 +9498,11 @@
           <t>Hattie McDaniel</t>
         </is>
       </c>
+      <c r="M58" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz, Mejor Actriz de Reparto, Mejor Guion Adaptado, Mejor Fotografía, Mejor Dirección Artística, Mejor Montaje, Premio Especial Técnico, Premio Honorífico</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -8761,6 +9555,11 @@
           <t>Ronald Lacey</t>
         </is>
       </c>
+      <c r="M59" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Dirección Artística, Mejor Montaje, Mejor Sonido, Mejores Efectos Visuales, Premio Especial Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n">
@@ -8813,6 +9612,11 @@
           <t>Joe Pantoliano</t>
         </is>
       </c>
+      <c r="M60" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -8865,6 +9669,11 @@
           <t>Yaphet Kotto</t>
         </is>
       </c>
+      <c r="M61" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n">
@@ -8917,6 +9726,11 @@
           <t>Elijah Wood</t>
         </is>
       </c>
+      <c r="M62" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -8969,6 +9783,11 @@
           <t>Thomas F. Wilson</t>
         </is>
       </c>
+      <c r="M63" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n">
@@ -9021,6 +9840,11 @@
           <t>Peter Boyle</t>
         </is>
       </c>
+      <c r="M64" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -9073,6 +9897,11 @@
           <t>Natascha McElhone</t>
         </is>
       </c>
+      <c r="M65" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n">
@@ -9125,6 +9954,11 @@
           <t>David Bowie</t>
         </is>
       </c>
+      <c r="M66" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -9177,6 +10011,11 @@
           <t>James Hong</t>
         </is>
       </c>
+      <c r="M67" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz, Mejor Actor de Reparto, Mejor Actriz de Reparto, Mejor Guion Original, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n">
@@ -9229,6 +10068,11 @@
           <t>Richard Harris</t>
         </is>
       </c>
+      <c r="M68" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor, Mejor Vestuario, Mejor Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -9281,6 +10125,11 @@
           <t>Mena Suvari</t>
         </is>
       </c>
+      <c r="M69" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Original, Mejor Fotografía</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n">
@@ -9333,6 +10182,11 @@
           <t>Matt Damon</t>
         </is>
       </c>
+      <c r="M70" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -9385,6 +10239,11 @@
           <t>Barry Nelson</t>
         </is>
       </c>
+      <c r="M71" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n">
@@ -9437,6 +10296,11 @@
           <t>Edward James Olmos</t>
         </is>
       </c>
+      <c r="M72" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -9489,6 +10353,11 @@
           <t>Adrienne Corri</t>
         </is>
       </c>
+      <c r="M73" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n">
@@ -9541,6 +10410,11 @@
           <t>Peter Appel</t>
         </is>
       </c>
+      <c r="M74" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -9593,6 +10467,11 @@
           <t>Dominique Pinon</t>
         </is>
       </c>
+      <c r="M75" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n">
@@ -9645,6 +10524,11 @@
           <t>Kelly Macdonald</t>
         </is>
       </c>
+      <c r="M76" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -9697,6 +10581,11 @@
           <t>Martin Sheen</t>
         </is>
       </c>
+      <c r="M77" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n">
@@ -9749,6 +10638,11 @@
           <t>Robert Loggia</t>
         </is>
       </c>
+      <c r="M78" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -9801,6 +10695,11 @@
           <t>Angus Macfadyen</t>
         </is>
       </c>
+      <c r="M79" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Fotografía, Mejor Edición de Sonido, Mejor Maquillaje</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n">
@@ -9853,6 +10752,11 @@
           <t>Willem Dafoe</t>
         </is>
       </c>
+      <c r="M80" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Banda Sonora, Mejor Diseño de Producción, Mejor Vestuario, Mejor Maquillaje y Peluquería</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -9905,6 +10809,11 @@
           <t>Peter Coyote</t>
         </is>
       </c>
+      <c r="M81" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n">
@@ -9957,6 +10866,11 @@
           <t>Murray Hamilton</t>
         </is>
       </c>
+      <c r="M82" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -10009,6 +10923,11 @@
           <t>Benedict Cumberbatch</t>
         </is>
       </c>
+      <c r="M83" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actriz de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n">
@@ -10061,6 +10980,11 @@
           <t>Dillon Freasier</t>
         </is>
       </c>
+      <c r="M84" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Fotografía</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -10113,6 +11037,11 @@
           <t>Samuel L. Jackson</t>
         </is>
       </c>
+      <c r="M85" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n">
@@ -10165,6 +11094,11 @@
           <t>Eli Roth</t>
         </is>
       </c>
+      <c r="M86" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Christoph Waltz)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -10217,6 +11151,11 @@
           <t>Arliss Howard</t>
         </is>
       </c>
+      <c r="M87" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n">
@@ -10269,6 +11208,11 @@
           <t>Rooney Mara</t>
         </is>
       </c>
+      <c r="M88" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Adaptado, Mejor Banda Sonora, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -10321,6 +11265,11 @@
           <t>Janelle Monáe</t>
         </is>
       </c>
+      <c r="M89" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n">
@@ -10373,6 +11322,11 @@
           <t>Rosemarie DeWitt</t>
         </is>
       </c>
+      <c r="M90" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actriz, Mejor Fotografía, Mejor Banda Sonora, Mejor Canción Original, Mejor Diseño de Producción</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -10425,6 +11379,11 @@
           <t>Bob Wells</t>
         </is>
       </c>
+      <c r="M91" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n">
@@ -10477,6 +11436,11 @@
           <t>Eli Wallach</t>
         </is>
       </c>
+      <c r="M92" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -10529,6 +11493,11 @@
           <t>Basher Savage</t>
         </is>
       </c>
+      <c r="M93" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Fotografía, Mejor Montaje, Mejores Efectos Visuales, Mejor Mezcla de Sonido, Mejor Edición de Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n">
@@ -10581,6 +11550,11 @@
           <t>Doug Jones</t>
         </is>
       </c>
+      <c r="M94" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Diseño de Producción, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -10633,7 +11607,13 @@
           <t>Forrest Goodluck</t>
         </is>
       </c>
-    </row>
+      <c r="M95" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actor, Mejor Fotografía</t>
+        </is>
+      </c>
+    </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
@@ -10658,7 +11638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M196"/>
+  <dimension ref="A1:N196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10674,6 +11654,7 @@
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="65" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -10756,6 +11737,11 @@
           <t>Fuente</t>
         </is>
       </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Categorías de Oscar</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -10813,6 +11799,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N5" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -10870,6 +11861,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N6" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion Adaptado, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -10927,6 +11923,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N7" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -10984,6 +11985,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N8" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje, Mejor Fotografía, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -11041,6 +12047,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -11098,6 +12109,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -11155,6 +12171,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N11" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -11212,6 +12233,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -11269,6 +12295,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N13" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -11328,6 +12359,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -11385,6 +12421,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Película de Habla No Inglesa, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -11442,6 +12483,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N16" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -11499,6 +12545,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N17" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Guion, Mejor Dirección Artística, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -11558,6 +12609,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N18" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -11615,6 +12671,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N19" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -11672,6 +12733,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N20" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Joe Pesci)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -11729,6 +12795,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N21" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -11786,6 +12857,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N22" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Dirección Artística, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -11843,6 +12919,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N23" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -11900,6 +12981,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N24" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -11959,6 +13045,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N25" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -12018,6 +13109,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N26" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion, Mejor Vestuario, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -12075,6 +13171,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N27" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -12132,6 +13233,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N28" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Maquillaje, Mejor Banda Sonora, Mejor Canción Original, Mejor Mezcla de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -12189,6 +13295,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N29" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Montaje, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -12246,6 +13357,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N30" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Sonido, Premio Especial Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -12303,6 +13419,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N31" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -12360,6 +13481,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N32" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Habla No Inglesa</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -12417,6 +13543,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N33" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
@@ -12474,6 +13605,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N34" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -12531,6 +13667,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N35" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
@@ -12588,6 +13729,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N36" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -12647,6 +13793,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N37" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Habla No Inglesa (Premio Honorífico)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -12704,6 +13855,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N38" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Heath Ledger), Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -12761,6 +13917,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N39" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actriz, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -12818,6 +13979,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N40" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Original, Mejor Película Internacional</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -12875,6 +14041,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N41" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -12932,6 +14103,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N42" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actor, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -12989,6 +14165,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N43" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actriz, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
@@ -13046,6 +14227,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N44" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -13103,6 +14289,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N45" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Dirección Artística, Mejor Vestuario, Mejor Maquillaje, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n">
@@ -13160,6 +14351,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N46" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Fotografía, Mejor Dirección Artística, Mejor Montaje, Mejor Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -13217,6 +14413,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N47" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
@@ -13274,6 +14475,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N48" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -13331,6 +14537,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N49" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n">
@@ -13388,6 +14599,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N50" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -13445,6 +14661,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N51" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Maquillaje, Mejor Banda Sonora, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
@@ -13502,6 +14723,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N52" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Mezcla de Sonido, Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -13559,6 +14785,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N53" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Dirección Artística, Mejor Vestuario, Mejor Sonido, Mejores Efectos Visuales, Mejor Banda Sonora, Premio Especial Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
@@ -13616,6 +14847,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N54" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido, Mejor Maquillaje</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -13673,6 +14909,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N55" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Fotografía, Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n">
@@ -13730,6 +14971,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N56" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -13787,6 +15033,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N57" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n">
@@ -13844,6 +15095,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N58" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Montaje, Mejor Mezcla de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -13901,6 +15157,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N59" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n">
@@ -13958,6 +15219,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N60" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Adaptado, Mejor Fotografía, Mejor Montaje, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -14015,6 +15281,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N61" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Banda Sonora, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n">
@@ -14072,6 +15343,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N62" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -14129,6 +15405,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N63" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz, Mejor Actriz de Reparto, Mejor Guion Adaptado, Mejor Fotografía, Mejor Dirección Artística, Mejor Montaje, Premio Especial Técnico, Premio Honorífico</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n">
@@ -14186,6 +15467,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N64" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Dirección Artística, Mejor Montaje, Mejor Sonido, Mejores Efectos Visuales, Premio Especial Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -14243,6 +15529,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N65" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n">
@@ -14300,6 +15591,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N66" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -14357,6 +15653,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N67" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n">
@@ -14414,6 +15715,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N68" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -14471,6 +15777,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N69" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actor de Reparto, Mejor Fotografía, Mejor Dirección Artística, Mejor Vestuario, Mejor Montaje, Mejor Sonido, Mejores Efectos Visuales, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n">
@@ -14528,6 +15839,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N70" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -14585,6 +15901,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N71" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n">
@@ -14642,6 +15963,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N72" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -14699,6 +16025,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N73" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n">
@@ -14756,6 +16087,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N74" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Actor de Reparto, Mejor Montaje, Mejor Fotografía, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -14813,6 +16149,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N75" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n">
@@ -14870,6 +16211,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N76" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor, Mejor Vestuario, Mejor Sonido, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -14927,6 +16273,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N77" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor, Mejor Guion Original, Mejor Fotografía</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n">
@@ -14984,6 +16335,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N78" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -15041,6 +16397,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N79" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz, Mejor Actor de Reparto, Mejor Actriz de Reparto, Mejor Guion Original, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n">
@@ -15098,6 +16459,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N80" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -15155,6 +16521,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N81" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n">
@@ -15212,6 +16583,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N82" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -15269,6 +16645,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N83" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n">
@@ -15326,6 +16707,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N84" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Montaje, Mejor Sonido, Mejor Edición de Sonido, Mejor Banda Sonora, Mejor Canción Original, Mejor Fotografía, Mejor Dirección Artística, Mejor Vestuario, Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -15383,6 +16769,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N85" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n">
@@ -15440,6 +16831,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N86" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Guion Adaptado, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -15497,6 +16893,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N87" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actor de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n">
@@ -15554,6 +16955,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N88" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -15611,6 +17017,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N89" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n">
@@ -15668,6 +17079,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N90" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales, Mejor Sonido, Mejor Edición de Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -15725,6 +17141,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N91" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Montaje, Mejor Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n">
@@ -15782,6 +17203,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N92" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto, Mejor Guion Original</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -15839,6 +17265,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N93" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor de Reparto (Christoph Waltz)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n">
@@ -15896,6 +17327,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N94" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Fotografía, Mejor Edición de Sonido, Mejor Maquillaje</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -15953,6 +17389,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N95" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actriz de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n">
@@ -16010,6 +17451,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N96" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Banda Sonora, Mejor Diseño de Producción, Mejor Vestuario, Mejor Maquillaje y Peluquería</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
@@ -16067,6 +17513,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N97" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Fotografía</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n">
@@ -16124,6 +17575,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N98" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -16181,6 +17637,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N99" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n">
@@ -16238,6 +17699,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N100" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
@@ -16295,6 +17761,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N101" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n">
@@ -16352,6 +17823,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N102" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Guion Adaptado, Mejor Banda Sonora, Mejor Montaje</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n">
@@ -16409,6 +17885,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N103" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Fotografía, Mejores Efectos Visuales, Mejor Dirección Artística</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="10" t="n">
@@ -16466,6 +17947,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N104" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n">
@@ -16523,6 +18009,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N105" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="n">
@@ -16580,6 +18071,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N106" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n">
@@ -16637,6 +18133,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N107" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n">
@@ -16694,6 +18195,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N108" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Actor, Mejor Montaje, Mejor Edición de Sonido, Mejor Mezcla de Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n">
@@ -16751,6 +18257,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N109" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Actor de Reparto, Mejor Guion Adaptado</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n">
@@ -16808,6 +18319,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N110" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n">
@@ -16865,6 +18381,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N111" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Sonido</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="10" t="n">
@@ -16922,6 +18443,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N112" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Edición de Sonido, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n">
@@ -16979,6 +18505,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N113" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actriz, Mejor Fotografía, Mejor Banda Sonora, Mejor Canción Original, Mejor Diseño de Producción</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="10" t="n">
@@ -17036,6 +18567,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N114" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Actriz</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n">
@@ -17093,6 +18629,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N115" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="10" t="n">
@@ -17150,6 +18691,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N116" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n">
@@ -17207,6 +18753,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N117" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="10" t="n">
@@ -17264,6 +18815,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N118" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n">
@@ -17321,6 +18877,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N119" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="10" t="n">
@@ -17378,6 +18939,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N120" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n">
@@ -17435,6 +19001,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N121" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="n">
@@ -17492,6 +19063,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N122" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n">
@@ -17549,6 +19125,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N123" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Fotografía, Mejor Montaje, Mejores Efectos Visuales, Mejor Mezcla de Sonido, Mejor Edición de Sonido, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="n">
@@ -17606,6 +19187,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N124" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Película, Mejor Director, Mejor Diseño de Producción, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n">
@@ -17663,6 +19249,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N125" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="n">
@@ -17720,6 +19311,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="N126" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Director, Mejor Actor, Mejor Fotografía</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n">
@@ -17777,6 +19373,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N127" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="n">
@@ -17834,6 +19435,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N128" s="27" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario, Mejor Diseño de Producción, Mejor Banda Sonora</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n">
@@ -17891,6 +19497,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N129" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="n">
@@ -17948,6 +19559,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N130" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n">
@@ -18005,6 +19621,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N131" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="10" t="n">
@@ -18062,6 +19683,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N132" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n">
@@ -18119,6 +19745,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N133" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="n">
@@ -18176,6 +19807,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N134" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n">
@@ -18233,6 +19869,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N135" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Película de Animación, Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="n">
@@ -18290,6 +19931,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N136" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n">
@@ -18347,6 +19993,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N137" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="10" t="n">
@@ -18404,6 +20055,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N138" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n">
@@ -18461,6 +20117,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N139" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="10" t="n">
@@ -18518,6 +20179,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N140" s="27" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n">
@@ -18575,6 +20241,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N141" s="25" t="inlineStr">
+        <is>
+          <t>Mejores Efectos Visuales</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="10" t="n">
@@ -18632,6 +20303,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N142" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n">
@@ -18689,6 +20365,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N143" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="10" t="n">
@@ -18746,6 +20427,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N144" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n">
@@ -18803,6 +20489,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N145" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="10" t="n">
@@ -18860,6 +20551,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N146" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n">
@@ -18917,6 +20613,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N147" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="10" t="n">
@@ -18974,6 +20675,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N148" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
@@ -19031,6 +20737,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N149" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="10" t="n">
@@ -19088,6 +20799,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N150" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n">
@@ -19145,6 +20861,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N151" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="10" t="n">
@@ -19202,6 +20923,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N152" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n">
@@ -19259,6 +20985,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N153" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="10" t="n">
@@ -19316,6 +21047,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N154" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n">
@@ -19373,6 +21109,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N155" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Canción Original</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="10" t="n">
@@ -19430,6 +21171,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N156" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n">
@@ -19487,6 +21233,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N157" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="10" t="n">
@@ -19544,6 +21295,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N158" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
@@ -19601,6 +21357,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N159" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="10" t="n">
@@ -19658,6 +21419,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N160" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n">
@@ -19715,6 +21481,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N161" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="10" t="n">
@@ -19772,6 +21543,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N162" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n">
@@ -19829,6 +21605,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N163" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="10" t="n">
@@ -19886,6 +21667,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N164" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n">
@@ -19943,6 +21729,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N165" s="25" t="inlineStr">
+        <is>
+          <t>Mejor Dirección Artística, Mejor Vestuario</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="10" t="n">
@@ -20000,6 +21791,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N166" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n">
@@ -20057,6 +21853,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N167" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="10" t="n">
@@ -20114,6 +21915,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N168" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
@@ -20171,6 +21977,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N169" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="10" t="n">
@@ -20228,6 +22039,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N170" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n">
@@ -20285,6 +22101,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N171" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="10" t="n">
@@ -20342,6 +22163,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N172" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n">
@@ -20399,6 +22225,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N173" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="10" t="n">
@@ -20456,6 +22287,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N174" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n">
@@ -20513,6 +22349,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N175" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="10" t="n">
@@ -20570,6 +22411,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N176" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n">
@@ -20627,6 +22473,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N177" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="10" t="n">
@@ -20684,6 +22535,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N178" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
@@ -20741,6 +22597,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N179" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="10" t="n">
@@ -20798,6 +22659,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N180" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n">
@@ -20855,6 +22721,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N181" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="10" t="n">
@@ -20912,6 +22783,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N182" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n">
@@ -20969,6 +22845,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N183" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="10" t="n">
@@ -21026,6 +22907,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N184" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n">
@@ -21085,6 +22971,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N185" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="10" t="n">
@@ -21144,6 +23035,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N186" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n">
@@ -21203,6 +23099,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N187" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="10" t="n">
@@ -21262,6 +23163,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N188" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n">
@@ -21321,6 +23227,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N189" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="10" t="n">
@@ -21380,6 +23291,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N190" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n">
@@ -21439,6 +23355,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N191" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="10" t="n">
@@ -21498,6 +23419,11 @@
           <t>Taquilla</t>
         </is>
       </c>
+      <c r="N192" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n">
@@ -21557,7 +23483,13 @@
           <t>Taquilla</t>
         </is>
       </c>
-    </row>
+      <c r="N193" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="194"/>
     <row r="195">
       <c r="A195" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Billions: datos regenerados con el Excel corregido
Notas de FilmAffinity actualizadas desde la última versión del archivo.
El Excel marca ahora como N/D la mayoría de las notas, así que las
películas del juego con nota utilizable bajan de 90 a 27 y las rondas de
crítica salen de un catálogo mucho más corto.

El resto de campos —director, reparto, Óscars y categorías— no cambia.

Incluye la lectura de hojas por nombre en tools/build-data.py: pedía
sheet3.xml a pelo, y ese nombre de archivo no tiene por qué corresponder
a la tercera pestaña; si se reordenan en Excel se leería otra hoja sin
avisar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/top_peliculas_taquilla_y_critica.xlsx
+++ b/top_peliculas_taquilla_y_critica.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,6 +93,12 @@
       <color rgb="00CCCCCC"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -154,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +229,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -706,7 +718,7 @@
         </is>
       </c>
       <c r="E5" s="8" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>3</v>
@@ -763,7 +775,7 @@
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>0</v>
@@ -820,7 +832,7 @@
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>1</v>
@@ -877,7 +889,7 @@
         </is>
       </c>
       <c r="E8" s="14" t="n">
-        <v>7.7</v>
+        <v>6.8</v>
       </c>
       <c r="F8" s="12" t="n">
         <v>11</v>
@@ -933,8 +945,10 @@
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
-        <v>6.8</v>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -1166,7 +1180,7 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -1281,8 +1295,10 @@
           <t>Kelsey Mann</t>
         </is>
       </c>
-      <c r="E15" s="8" t="n">
-        <v>7</v>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F15" s="6" t="n">
         <v>1</v>
@@ -1339,7 +1355,7 @@
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="F16" s="12" t="n">
         <v>0</v>
@@ -1395,8 +1411,10 @@
           <t>Jon Favreau</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
-        <v>6.3</v>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -1453,7 +1471,7 @@
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="F18" s="12" t="n">
         <v>0</v>
@@ -1509,8 +1527,10 @@
           <t>James Wan</t>
         </is>
       </c>
-      <c r="E19" s="8" t="n">
-        <v>6.2</v>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
@@ -1566,10 +1586,8 @@
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
+      <c r="E20" s="14" t="n">
+        <v>6.3</v>
       </c>
       <c r="F20" s="12" t="n">
         <v>0</v>
@@ -1625,8 +1643,10 @@
           <t>Joseph Kosinski</t>
         </is>
       </c>
-      <c r="E21" s="8" t="n">
-        <v>7.2</v>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F21" s="6" t="n">
         <v>1</v>
@@ -1682,8 +1702,10 @@
           <t>Chris Buck &amp; Jennifer Lee</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>5.9</v>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F22" s="12" t="n">
         <v>0</v>
@@ -1739,8 +1761,10 @@
           <t>Greta Gerwig</t>
         </is>
       </c>
-      <c r="E23" s="8" t="n">
-        <v>6.5</v>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F23" s="6" t="n">
         <v>1</v>
@@ -1797,7 +1821,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="F24" s="12" t="n">
         <v>0</v>
@@ -1853,8 +1877,10 @@
           <t>Aaron Horvath &amp; Michael Jelenic</t>
         </is>
       </c>
-      <c r="E25" s="8" t="n">
-        <v>6</v>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F25" s="6" t="n">
         <v>0</v>
@@ -1969,8 +1995,10 @@
           <t>Shawn Levy</t>
         </is>
       </c>
-      <c r="E27" s="8" t="n">
-        <v>7</v>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F27" s="6" t="n">
         <v>0</v>
@@ -2027,7 +2055,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="F28" s="12" t="n">
         <v>3</v>
@@ -2083,8 +2111,10 @@
           <t>Rian Johnson</t>
         </is>
       </c>
-      <c r="E29" s="8" t="n">
-        <v>6</v>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F29" s="6" t="n">
         <v>0</v>
@@ -2140,8 +2170,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>7.4</v>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F30" s="12" t="n">
         <v>0</v>
@@ -2254,8 +2286,10 @@
           <t>Chris Buck &amp; Jennifer Lee</t>
         </is>
       </c>
-      <c r="E32" s="14" t="n">
-        <v>6.7</v>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F32" s="12" t="n">
         <v>2</v>
@@ -2311,8 +2345,10 @@
           <t>Bill Condon</t>
         </is>
       </c>
-      <c r="E33" s="8" t="n">
-        <v>6.4</v>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -2368,8 +2404,10 @@
           <t>Brad Bird</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>6.8</v>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F34" s="12" t="n">
         <v>0</v>
@@ -2426,7 +2464,7 @@
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -2482,8 +2520,10 @@
           <t>F. Gary Gray</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>5.4</v>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F36" s="12" t="n">
         <v>0</v>
@@ -2539,8 +2579,10 @@
           <t>Pierre Coffin &amp; Kyle Balda</t>
         </is>
       </c>
-      <c r="E37" s="8" t="n">
-        <v>5.4</v>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
@@ -2597,7 +2639,7 @@
         </is>
       </c>
       <c r="E38" s="14" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>0</v>
@@ -2653,8 +2695,10 @@
           <t>James Wan</t>
         </is>
       </c>
-      <c r="E39" s="8" t="n">
-        <v>5.8</v>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F39" s="6" t="n">
         <v>0</v>
@@ -2711,7 +2755,7 @@
         </is>
       </c>
       <c r="E40" s="14" t="n">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>0</v>
@@ -2768,7 +2812,7 @@
         </is>
       </c>
       <c r="E41" s="8" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
@@ -2881,8 +2925,10 @@
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="E43" s="8" t="n">
-        <v>5.2</v>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F43" s="6" t="n">
         <v>0</v>
@@ -2997,8 +3043,10 @@
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="E45" s="8" t="n">
-        <v>7.2</v>
+      <c r="E45" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F45" s="6" t="n">
         <v>2</v>
@@ -3054,8 +3102,10 @@
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="E46" s="14" t="n">
-        <v>4.5</v>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F46" s="12" t="n">
         <v>0</v>
@@ -3111,8 +3161,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>7.5</v>
+      <c r="E47" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F47" s="6" t="n">
         <v>0</v>
@@ -3168,8 +3220,10 @@
           <t>Todd Phillips</t>
         </is>
       </c>
-      <c r="E48" s="14" t="n">
-        <v>7.5</v>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F48" s="12" t="n">
         <v>2</v>
@@ -3225,8 +3279,10 @@
           <t>Josh Cooley</t>
         </is>
       </c>
-      <c r="E49" s="8" t="n">
-        <v>7.1</v>
+      <c r="E49" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F49" s="6" t="n">
         <v>1</v>
@@ -3282,8 +3338,10 @@
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="E50" s="14" t="n">
-        <v>5.5</v>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F50" s="12" t="n">
         <v>0</v>
@@ -3339,8 +3397,10 @@
           <t>Lee Unkrich</t>
         </is>
       </c>
-      <c r="E51" s="8" t="n">
-        <v>7.8</v>
+      <c r="E51" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F51" s="6" t="n">
         <v>2</v>
@@ -3396,8 +3456,10 @@
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="E52" s="14" t="n">
-        <v>6.6</v>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F52" s="12" t="n">
         <v>1</v>
@@ -3453,8 +3515,10 @@
           <t>David Derrick Jr.</t>
         </is>
       </c>
-      <c r="E53" s="8" t="n">
-        <v>5.5</v>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F53" s="6" t="n">
         <v>0</v>
@@ -3511,7 +3575,7 @@
         </is>
       </c>
       <c r="E54" s="14" t="n">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
       <c r="F54" s="12" t="n">
         <v>3</v>
@@ -3567,8 +3631,10 @@
           <t>Gareth Edwards</t>
         </is>
       </c>
-      <c r="E55" s="8" t="n">
-        <v>6.8</v>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F55" s="6" t="n">
         <v>0</v>
@@ -3624,8 +3690,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E56" s="14" t="n">
-        <v>5.8</v>
+      <c r="E56" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F56" s="12" t="n">
         <v>0</v>
@@ -3681,8 +3749,10 @@
           <t>Rob Marshall</t>
         </is>
       </c>
-      <c r="E57" s="8" t="n">
-        <v>5.4</v>
+      <c r="E57" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F57" s="6" t="n">
         <v>0</v>
@@ -3738,8 +3808,10 @@
           <t>Guy Ritchie</t>
         </is>
       </c>
-      <c r="E58" s="14" t="n">
-        <v>6.1</v>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F58" s="12" t="n">
         <v>0</v>
@@ -3854,8 +3926,10 @@
           <t>Pierre Coffin &amp; Kyle Balda</t>
         </is>
       </c>
-      <c r="E60" s="14" t="n">
-        <v>5.5</v>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F60" s="12" t="n">
         <v>0</v>
@@ -3911,8 +3985,10 @@
           <t>Tim Burton</t>
         </is>
       </c>
-      <c r="E61" s="8" t="n">
-        <v>5.8</v>
+      <c r="E61" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F61" s="6" t="n">
         <v>2</v>
@@ -3968,8 +4044,10 @@
           <t>Andrew Stanton</t>
         </is>
       </c>
-      <c r="E62" s="14" t="n">
-        <v>6.6</v>
+      <c r="E62" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F62" s="12" t="n">
         <v>0</v>
@@ -4025,8 +4103,10 @@
           <t>Byron Howard &amp; Rich Moore</t>
         </is>
       </c>
-      <c r="E63" s="8" t="n">
-        <v>7.4</v>
+      <c r="E63" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F63" s="6" t="n">
         <v>1</v>
@@ -4082,8 +4162,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E64" s="14" t="n">
-        <v>6.6</v>
+      <c r="E64" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F64" s="12" t="n">
         <v>0</v>
@@ -4310,8 +4392,10 @@
           <t>Chris Renaud</t>
         </is>
       </c>
-      <c r="E68" s="14" t="n">
-        <v>5.6</v>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F68" s="12" t="n">
         <v>0</v>
@@ -4367,8 +4451,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E69" s="8" t="n">
-        <v>7.8</v>
+      <c r="E69" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F69" s="6" t="n">
         <v>7</v>
@@ -4424,8 +4510,10 @@
           <t>Pierre Coffin &amp; Chris Renaud</t>
         </is>
       </c>
-      <c r="E70" s="14" t="n">
-        <v>6.2</v>
+      <c r="E70" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F70" s="12" t="n">
         <v>0</v>
@@ -4481,8 +4569,10 @@
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="E71" s="8" t="n">
-        <v>7.3</v>
+      <c r="E71" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F71" s="6" t="n">
         <v>0</v>
@@ -4538,8 +4628,10 @@
           <t>Jake Kasdan</t>
         </is>
       </c>
-      <c r="E72" s="14" t="n">
-        <v>6.2</v>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F72" s="12" t="n">
         <v>0</v>
@@ -4654,8 +4746,10 @@
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="E74" s="14" t="n">
-        <v>6</v>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F74" s="12" t="n">
         <v>0</v>
@@ -4711,8 +4805,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E75" s="8" t="n">
-        <v>6.6</v>
+      <c r="E75" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F75" s="6" t="n">
         <v>0</v>
@@ -4769,7 +4865,7 @@
         </is>
       </c>
       <c r="E76" s="14" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="F76" s="12" t="n">
         <v>0</v>
@@ -4825,8 +4921,10 @@
           <t>Jon Favreau</t>
         </is>
       </c>
-      <c r="E77" s="8" t="n">
-        <v>6.8</v>
+      <c r="E77" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F77" s="6" t="n">
         <v>1</v>
@@ -4882,8 +4980,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E78" s="14" t="n">
-        <v>7</v>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F78" s="12" t="n">
         <v>0</v>
@@ -4939,8 +5039,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E79" s="8" t="n">
-        <v>6.1</v>
+      <c r="E79" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F79" s="6" t="n">
         <v>0</v>
@@ -4996,8 +5098,10 @@
           <t>Kyle Balda</t>
         </is>
       </c>
-      <c r="E80" s="14" t="n">
-        <v>5.7</v>
+      <c r="E80" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F80" s="12" t="n">
         <v>0</v>
@@ -5053,8 +5157,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E81" s="8" t="n">
-        <v>6.8</v>
+      <c r="E81" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F81" s="6" t="n">
         <v>0</v>
@@ -5110,8 +5216,10 @@
           <t>Andrew Stanton</t>
         </is>
       </c>
-      <c r="E82" s="14" t="n">
-        <v>7.7</v>
+      <c r="E82" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F82" s="12" t="n">
         <v>1</v>
@@ -5167,8 +5275,10 @@
           <t>Andrew Adamson</t>
         </is>
       </c>
-      <c r="E83" s="8" t="n">
-        <v>6.8</v>
+      <c r="E83" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F83" s="6" t="n">
         <v>0</v>
@@ -5281,8 +5391,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E85" s="8" t="n">
-        <v>6.8</v>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F85" s="6" t="n">
         <v>0</v>
@@ -5338,8 +5450,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E86" s="14" t="n">
-        <v>6.7</v>
+      <c r="E86" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F86" s="12" t="n">
         <v>0</v>
@@ -5452,8 +5566,10 @@
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="E88" s="14" t="n">
-        <v>5.5</v>
+      <c r="E88" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F88" s="12" t="n">
         <v>0</v>
@@ -5509,8 +5625,10 @@
           <t>Mike Newell</t>
         </is>
       </c>
-      <c r="E89" s="8" t="n">
-        <v>7</v>
+      <c r="E89" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F89" s="6" t="n">
         <v>0</v>
@@ -5566,8 +5684,10 @@
           <t>Carlos Saldanha</t>
         </is>
       </c>
-      <c r="E90" s="14" t="n">
-        <v>5.8</v>
+      <c r="E90" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F90" s="12" t="n">
         <v>0</v>
@@ -5623,8 +5743,10 @@
           <t>Chris Renaud</t>
         </is>
       </c>
-      <c r="E91" s="8" t="n">
-        <v>5.7</v>
+      <c r="E91" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F91" s="6" t="n">
         <v>0</v>
@@ -5680,8 +5802,10 @@
           <t>Steve Martino</t>
         </is>
       </c>
-      <c r="E92" s="14" t="n">
-        <v>5</v>
+      <c r="E92" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F92" s="12" t="n">
         <v>0</v>
@@ -5737,8 +5861,10 @@
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="E93" s="8" t="n">
-        <v>7.3</v>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F93" s="6" t="n">
         <v>4</v>
@@ -5794,8 +5920,10 @@
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="E94" s="14" t="n">
-        <v>6.1</v>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F94" s="12" t="n">
         <v>1</v>
@@ -5852,7 +5980,7 @@
         </is>
       </c>
       <c r="E95" s="8" t="n">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="F95" s="6" t="n">
         <v>0</v>
@@ -5908,8 +6036,10 @@
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="E96" s="14" t="n">
-        <v>7.1</v>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F96" s="12" t="n">
         <v>0</v>
@@ -5965,8 +6095,10 @@
           <t>Zack Snyder</t>
         </is>
       </c>
-      <c r="E97" s="8" t="n">
-        <v>5.5</v>
+      <c r="E97" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F97" s="6" t="n">
         <v>0</v>
@@ -6082,7 +6214,7 @@
         </is>
       </c>
       <c r="E99" s="8" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="F99" s="6" t="n">
         <v>0</v>
@@ -6138,8 +6270,10 @@
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="E100" s="14" t="n">
-        <v>6.7</v>
+      <c r="E100" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F100" s="12" t="n">
         <v>0</v>
@@ -6196,7 +6330,7 @@
         </is>
       </c>
       <c r="E101" s="8" t="n">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="F101" s="6" t="n">
         <v>1</v>
@@ -6252,8 +6386,10 @@
           <t>Ruben Fleischer</t>
         </is>
       </c>
-      <c r="E102" s="14" t="n">
-        <v>5.4</v>
+      <c r="E102" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F102" s="12" t="n">
         <v>0</v>
@@ -7695,8 +7831,10 @@
           <t>Alfred Hitchcock</t>
         </is>
       </c>
-      <c r="E27" s="8" t="n">
-        <v>8.300000000000001</v>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F27" s="6" t="n">
         <v>0</v>
@@ -7809,8 +7947,10 @@
           <t>Irvin Kershner</t>
         </is>
       </c>
-      <c r="E29" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F29" s="6" t="n">
         <v>2</v>
@@ -7866,8 +8006,10 @@
           <t>Orson Welles</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F30" s="12" t="n">
         <v>1</v>
@@ -7923,8 +8065,10 @@
           <t>Hayao Miyazaki</t>
         </is>
       </c>
-      <c r="E31" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F31" s="6" t="n">
         <v>1</v>
@@ -7980,8 +8124,10 @@
           <t>Giuseppe Tornatore</t>
         </is>
       </c>
-      <c r="E32" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F32" s="12" t="n">
         <v>1</v>
@@ -8037,8 +8183,10 @@
           <t>Akira Kurosawa</t>
         </is>
       </c>
-      <c r="E33" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F33" s="6" t="n">
         <v>1</v>
@@ -8096,8 +8244,10 @@
           <t>Alfred Hitchcock</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F34" s="12" t="n">
         <v>0</v>
@@ -8153,8 +8303,10 @@
           <t>Stanley Donen &amp; Gene Kelly</t>
         </is>
       </c>
-      <c r="E35" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -8210,8 +8362,10 @@
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F36" s="12" t="n">
         <v>0</v>
@@ -8267,8 +8421,10 @@
           <t>Miloš Forman</t>
         </is>
       </c>
-      <c r="E37" s="8" t="n">
-        <v>8.1</v>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F37" s="6" t="n">
         <v>8</v>
@@ -8324,8 +8480,10 @@
           <t>David Lean</t>
         </is>
       </c>
-      <c r="E38" s="14" t="n">
-        <v>8.1</v>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F38" s="12" t="n">
         <v>7</v>
@@ -8382,7 +8540,7 @@
         </is>
       </c>
       <c r="E39" s="8" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>5</v>
@@ -8438,8 +8596,10 @@
           <t>Miloš Forman</t>
         </is>
       </c>
-      <c r="E40" s="14" t="n">
-        <v>8.1</v>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F40" s="12" t="n">
         <v>5</v>
@@ -8495,8 +8655,10 @@
           <t>Bong Joon-ho</t>
         </is>
       </c>
-      <c r="E41" s="8" t="n">
-        <v>8.1</v>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F41" s="6" t="n">
         <v>4</v>
@@ -8552,8 +8714,10 @@
           <t>Roman Polanski</t>
         </is>
       </c>
-      <c r="E42" s="14" t="n">
-        <v>8.1</v>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F42" s="12" t="n">
         <v>3</v>
@@ -8609,8 +8773,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E43" s="8" t="n">
-        <v>8.1</v>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F43" s="6" t="n">
         <v>2</v>
@@ -8666,8 +8832,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E44" s="14" t="n">
-        <v>8.1</v>
+      <c r="E44" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F44" s="12" t="n">
         <v>1</v>
@@ -8723,8 +8891,10 @@
           <t>Billy Wilder</t>
         </is>
       </c>
-      <c r="E45" s="8" t="n">
-        <v>8.1</v>
+      <c r="E45" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F45" s="6" t="n">
         <v>1</v>
@@ -8837,8 +9007,10 @@
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>8.1</v>
+      <c r="E47" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F47" s="6" t="n">
         <v>0</v>
@@ -8894,8 +9066,10 @@
           <t>David Lean</t>
         </is>
       </c>
-      <c r="E48" s="14" t="n">
-        <v>8</v>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F48" s="12" t="n">
         <v>7</v>
@@ -8951,8 +9125,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E49" s="8" t="n">
-        <v>8</v>
+      <c r="E49" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F49" s="6" t="n">
         <v>7</v>
@@ -9008,8 +9184,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E50" s="14" t="n">
-        <v>8</v>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F50" s="12" t="n">
         <v>5</v>
@@ -9122,8 +9300,10 @@
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="E52" s="14" t="n">
-        <v>8</v>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F52" s="12" t="n">
         <v>4</v>
@@ -9179,8 +9359,10 @@
           <t>Damien Chazelle</t>
         </is>
       </c>
-      <c r="E53" s="8" t="n">
-        <v>8</v>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F53" s="6" t="n">
         <v>3</v>
@@ -9236,8 +9418,10 @@
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="E54" s="14" t="n">
-        <v>8</v>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F54" s="12" t="n">
         <v>2</v>
@@ -9293,8 +9477,10 @@
           <t>Francis Ford Coppola</t>
         </is>
       </c>
-      <c r="E55" s="8" t="n">
-        <v>8</v>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F55" s="6" t="n">
         <v>2</v>
@@ -9350,8 +9536,10 @@
           <t>Frank Darabont</t>
         </is>
       </c>
-      <c r="E56" s="14" t="n">
-        <v>8</v>
+      <c r="E56" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F56" s="12" t="n">
         <v>0</v>
@@ -9407,8 +9595,10 @@
           <t>William Wyler</t>
         </is>
       </c>
-      <c r="E57" s="8" t="n">
-        <v>7.9</v>
+      <c r="E57" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F57" s="6" t="n">
         <v>11</v>
@@ -9464,8 +9654,10 @@
           <t>Victor Fleming</t>
         </is>
       </c>
-      <c r="E58" s="14" t="n">
-        <v>7.9</v>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F58" s="12" t="n">
         <v>10</v>
@@ -9521,8 +9713,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E59" s="8" t="n">
-        <v>7.9</v>
+      <c r="E59" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F59" s="6" t="n">
         <v>5</v>
@@ -9635,8 +9829,10 @@
           <t>Ridley Scott</t>
         </is>
       </c>
-      <c r="E61" s="8" t="n">
-        <v>7.9</v>
+      <c r="E61" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F61" s="6" t="n">
         <v>1</v>
@@ -9692,8 +9888,10 @@
           <t>Michel Gondry</t>
         </is>
       </c>
-      <c r="E62" s="14" t="n">
-        <v>7.9</v>
+      <c r="E62" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F62" s="12" t="n">
         <v>1</v>
@@ -9749,8 +9947,10 @@
           <t>Robert Zemeckis</t>
         </is>
       </c>
-      <c r="E63" s="8" t="n">
-        <v>7.9</v>
+      <c r="E63" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F63" s="6" t="n">
         <v>1</v>
@@ -9806,8 +10006,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E64" s="14" t="n">
-        <v>7.9</v>
+      <c r="E64" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F64" s="12" t="n">
         <v>0</v>
@@ -9863,8 +10065,10 @@
           <t>Peter Weir</t>
         </is>
       </c>
-      <c r="E65" s="8" t="n">
-        <v>7.9</v>
+      <c r="E65" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F65" s="6" t="n">
         <v>0</v>
@@ -9920,8 +10124,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E66" s="14" t="n">
-        <v>7.9</v>
+      <c r="E66" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F66" s="12" t="n">
         <v>0</v>
@@ -9977,8 +10183,10 @@
           <t>Daniel Kwan &amp; Daniel Scheinert</t>
         </is>
       </c>
-      <c r="E67" s="8" t="n">
-        <v>7.8</v>
+      <c r="E67" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F67" s="6" t="n">
         <v>7</v>
@@ -10035,7 +10243,7 @@
         </is>
       </c>
       <c r="E68" s="14" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F68" s="12" t="n">
         <v>5</v>
@@ -10092,7 +10300,7 @@
         </is>
       </c>
       <c r="E69" s="8" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F69" s="6" t="n">
         <v>5</v>
@@ -10148,8 +10356,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E70" s="14" t="n">
-        <v>7.8</v>
+      <c r="E70" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F70" s="12" t="n">
         <v>1</v>
@@ -10205,8 +10415,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E71" s="8" t="n">
-        <v>7.8</v>
+      <c r="E71" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F71" s="6" t="n">
         <v>0</v>
@@ -10262,8 +10474,10 @@
           <t>Ridley Scott</t>
         </is>
       </c>
-      <c r="E72" s="14" t="n">
-        <v>7.8</v>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F72" s="12" t="n">
         <v>0</v>
@@ -10320,7 +10534,7 @@
         </is>
       </c>
       <c r="E73" s="8" t="n">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F73" s="6" t="n">
         <v>0</v>
@@ -10376,8 +10590,10 @@
           <t>Luc Besson</t>
         </is>
       </c>
-      <c r="E74" s="14" t="n">
-        <v>7.8</v>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F74" s="12" t="n">
         <v>0</v>
@@ -10490,8 +10706,10 @@
           <t>Joel &amp; Ethan Coen</t>
         </is>
       </c>
-      <c r="E76" s="14" t="n">
-        <v>7.7</v>
+      <c r="E76" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F76" s="12" t="n">
         <v>4</v>
@@ -10547,8 +10765,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E77" s="8" t="n">
-        <v>7.7</v>
+      <c r="E77" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F77" s="6" t="n">
         <v>4</v>
@@ -10604,8 +10824,10 @@
           <t>Brian De Palma</t>
         </is>
       </c>
-      <c r="E78" s="14" t="n">
-        <v>7.7</v>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F78" s="12" t="n">
         <v>0</v>
@@ -10661,8 +10883,10 @@
           <t>Mel Gibson</t>
         </is>
       </c>
-      <c r="E79" s="8" t="n">
-        <v>7.6</v>
+      <c r="E79" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F79" s="6" t="n">
         <v>5</v>
@@ -10718,8 +10942,10 @@
           <t>Wes Anderson</t>
         </is>
       </c>
-      <c r="E80" s="14" t="n">
-        <v>7.6</v>
+      <c r="E80" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F80" s="12" t="n">
         <v>4</v>
@@ -10775,8 +11001,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E81" s="8" t="n">
-        <v>7.6</v>
+      <c r="E81" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F81" s="6" t="n">
         <v>4</v>
@@ -10832,8 +11060,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E82" s="14" t="n">
-        <v>7.6</v>
+      <c r="E82" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F82" s="12" t="n">
         <v>3</v>
@@ -10889,8 +11119,10 @@
           <t>Steve McQueen</t>
         </is>
       </c>
-      <c r="E83" s="8" t="n">
-        <v>7.6</v>
+      <c r="E83" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F83" s="6" t="n">
         <v>3</v>
@@ -10946,8 +11178,10 @@
           <t>Paul Thomas Anderson</t>
         </is>
       </c>
-      <c r="E84" s="14" t="n">
-        <v>7.6</v>
+      <c r="E84" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F84" s="12" t="n">
         <v>2</v>
@@ -11003,8 +11237,10 @@
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="E85" s="8" t="n">
-        <v>7.6</v>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F85" s="6" t="n">
         <v>2</v>
@@ -11061,7 +11297,7 @@
         </is>
       </c>
       <c r="E86" s="14" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="F86" s="12" t="n">
         <v>1</v>
@@ -11117,8 +11353,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E87" s="8" t="n">
-        <v>7.6</v>
+      <c r="E87" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F87" s="6" t="n">
         <v>0</v>
@@ -11174,8 +11412,10 @@
           <t>David Fincher</t>
         </is>
       </c>
-      <c r="E88" s="14" t="n">
-        <v>7.5</v>
+      <c r="E88" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F88" s="12" t="n">
         <v>3</v>
@@ -11231,8 +11471,10 @@
           <t>Barry Jenkins</t>
         </is>
       </c>
-      <c r="E89" s="8" t="n">
-        <v>7.3</v>
+      <c r="E89" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F89" s="6" t="n">
         <v>3</v>
@@ -11288,8 +11530,10 @@
           <t>Damien Chazelle</t>
         </is>
       </c>
-      <c r="E90" s="14" t="n">
-        <v>7.2</v>
+      <c r="E90" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F90" s="12" t="n">
         <v>6</v>
@@ -11345,8 +11589,10 @@
           <t>Chloé Zhao</t>
         </is>
       </c>
-      <c r="E91" s="8" t="n">
-        <v>7.2</v>
+      <c r="E91" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F91" s="6" t="n">
         <v>3</v>
@@ -11402,8 +11648,10 @@
           <t>Francis Ford Coppola</t>
         </is>
       </c>
-      <c r="E92" s="14" t="n">
-        <v>7.1</v>
+      <c r="E92" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F92" s="12" t="n">
         <v>0</v>
@@ -11459,8 +11707,10 @@
           <t>Alfonso Cuarón</t>
         </is>
       </c>
-      <c r="E93" s="8" t="n">
-        <v>7</v>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F93" s="6" t="n">
         <v>7</v>
@@ -11516,8 +11766,10 @@
           <t>Guillermo del Toro</t>
         </is>
       </c>
-      <c r="E94" s="14" t="n">
-        <v>7</v>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F94" s="12" t="n">
         <v>4</v>
@@ -11573,8 +11825,10 @@
           <t>Alejandro G. Iñárritu</t>
         </is>
       </c>
-      <c r="E95" s="8" t="n">
-        <v>6.9</v>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F95" s="6" t="n">
         <v>3</v>
@@ -13132,8 +13386,10 @@
           <t>Alfred Hitchcock</t>
         </is>
       </c>
-      <c r="E27" s="8" t="n">
-        <v>8.300000000000001</v>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F27" s="6" t="n">
         <v>0</v>
@@ -13318,8 +13574,10 @@
           <t>Irvin Kershner</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F30" s="12" t="n">
         <v>2</v>
@@ -13380,8 +13638,10 @@
           <t>Hayao Miyazaki</t>
         </is>
       </c>
-      <c r="E31" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F31" s="6" t="n">
         <v>1</v>
@@ -13442,8 +13702,10 @@
           <t>Giuseppe Tornatore</t>
         </is>
       </c>
-      <c r="E32" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F32" s="12" t="n">
         <v>1</v>
@@ -13504,8 +13766,10 @@
           <t>Stanley Donen &amp; Gene Kelly</t>
         </is>
       </c>
-      <c r="E33" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -13566,8 +13830,10 @@
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F34" s="12" t="n">
         <v>0</v>
@@ -13628,8 +13894,10 @@
           <t>Alfred Hitchcock</t>
         </is>
       </c>
-      <c r="E35" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -13690,8 +13958,10 @@
           <t>Orson Welles</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>8.199999999999999</v>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F36" s="12" t="n">
         <v>1</v>
@@ -13752,8 +14022,10 @@
           <t>Akira Kurosawa</t>
         </is>
       </c>
-      <c r="E37" s="8" t="n">
-        <v>8.199999999999999</v>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F37" s="6" t="n">
         <v>1</v>
@@ -13879,7 +14151,7 @@
         </is>
       </c>
       <c r="E39" s="8" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>5</v>
@@ -13940,8 +14212,10 @@
           <t>Bong Joon-ho</t>
         </is>
       </c>
-      <c r="E40" s="14" t="n">
-        <v>8.1</v>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F40" s="12" t="n">
         <v>4</v>
@@ -14002,8 +14276,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E41" s="8" t="n">
-        <v>8.1</v>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F41" s="6" t="n">
         <v>1</v>
@@ -14064,8 +14340,10 @@
           <t>Roman Polanski</t>
         </is>
       </c>
-      <c r="E42" s="14" t="n">
-        <v>8.1</v>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F42" s="12" t="n">
         <v>3</v>
@@ -14126,8 +14404,10 @@
           <t>Miloš Forman</t>
         </is>
       </c>
-      <c r="E43" s="8" t="n">
-        <v>8.1</v>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F43" s="6" t="n">
         <v>5</v>
@@ -14250,8 +14530,10 @@
           <t>Miloš Forman</t>
         </is>
       </c>
-      <c r="E45" s="8" t="n">
-        <v>8.1</v>
+      <c r="E45" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F45" s="6" t="n">
         <v>8</v>
@@ -14312,8 +14594,10 @@
           <t>David Lean</t>
         </is>
       </c>
-      <c r="E46" s="14" t="n">
-        <v>8.1</v>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F46" s="12" t="n">
         <v>7</v>
@@ -14374,8 +14658,10 @@
           <t>Billy Wilder</t>
         </is>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>8.1</v>
+      <c r="E47" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F47" s="6" t="n">
         <v>1</v>
@@ -14436,8 +14722,10 @@
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="E48" s="14" t="n">
-        <v>8.1</v>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F48" s="12" t="n">
         <v>0</v>
@@ -14498,8 +14786,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E49" s="8" t="n">
-        <v>8.1</v>
+      <c r="E49" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F49" s="6" t="n">
         <v>2</v>
@@ -14746,8 +15036,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E53" s="8" t="n">
-        <v>8</v>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F53" s="6" t="n">
         <v>7</v>
@@ -14808,8 +15100,10 @@
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="E54" s="14" t="n">
-        <v>8</v>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F54" s="12" t="n">
         <v>4</v>
@@ -14870,8 +15164,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E55" s="8" t="n">
-        <v>8</v>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F55" s="6" t="n">
         <v>5</v>
@@ -14932,8 +15228,10 @@
           <t>Frank Darabont</t>
         </is>
       </c>
-      <c r="E56" s="14" t="n">
-        <v>8</v>
+      <c r="E56" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F56" s="12" t="n">
         <v>0</v>
@@ -14994,8 +15292,10 @@
           <t>Francis Ford Coppola</t>
         </is>
       </c>
-      <c r="E57" s="8" t="n">
-        <v>8</v>
+      <c r="E57" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F57" s="6" t="n">
         <v>2</v>
@@ -15056,8 +15356,10 @@
           <t>Damien Chazelle</t>
         </is>
       </c>
-      <c r="E58" s="14" t="n">
-        <v>8</v>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F58" s="12" t="n">
         <v>3</v>
@@ -15118,8 +15420,10 @@
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="E59" s="8" t="n">
-        <v>8</v>
+      <c r="E59" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F59" s="6" t="n">
         <v>2</v>
@@ -15180,8 +15484,10 @@
           <t>David Lean</t>
         </is>
       </c>
-      <c r="E60" s="14" t="n">
-        <v>8</v>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F60" s="12" t="n">
         <v>7</v>
@@ -15366,8 +15672,10 @@
           <t>Victor Fleming</t>
         </is>
       </c>
-      <c r="E63" s="8" t="n">
-        <v>7.9</v>
+      <c r="E63" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F63" s="6" t="n">
         <v>10</v>
@@ -15428,8 +15736,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E64" s="14" t="n">
-        <v>7.9</v>
+      <c r="E64" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F64" s="12" t="n">
         <v>5</v>
@@ -15490,8 +15800,10 @@
           <t>Robert Zemeckis</t>
         </is>
       </c>
-      <c r="E65" s="8" t="n">
-        <v>7.9</v>
+      <c r="E65" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F65" s="6" t="n">
         <v>1</v>
@@ -15552,8 +15864,10 @@
           <t>Peter Weir</t>
         </is>
       </c>
-      <c r="E66" s="14" t="n">
-        <v>7.9</v>
+      <c r="E66" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F66" s="12" t="n">
         <v>0</v>
@@ -15614,8 +15928,10 @@
           <t>Ridley Scott</t>
         </is>
       </c>
-      <c r="E67" s="8" t="n">
-        <v>7.9</v>
+      <c r="E67" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F67" s="6" t="n">
         <v>1</v>
@@ -15676,8 +15992,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E68" s="14" t="n">
-        <v>7.9</v>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F68" s="12" t="n">
         <v>0</v>
@@ -15738,8 +16056,10 @@
           <t>William Wyler</t>
         </is>
       </c>
-      <c r="E69" s="8" t="n">
-        <v>7.9</v>
+      <c r="E69" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F69" s="6" t="n">
         <v>11</v>
@@ -15800,8 +16120,10 @@
           <t>Michel Gondry</t>
         </is>
       </c>
-      <c r="E70" s="14" t="n">
-        <v>7.9</v>
+      <c r="E70" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F70" s="12" t="n">
         <v>1</v>
@@ -15862,8 +16184,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E71" s="8" t="n">
-        <v>7.9</v>
+      <c r="E71" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F71" s="6" t="n">
         <v>0</v>
@@ -15924,8 +16248,10 @@
           <t>Lee Unkrich</t>
         </is>
       </c>
-      <c r="E72" s="14" t="n">
-        <v>7.8</v>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F72" s="12" t="n">
         <v>2</v>
@@ -15987,7 +16313,7 @@
         </is>
       </c>
       <c r="E73" s="8" t="n">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
       <c r="F73" s="6" t="n">
         <v>3</v>
@@ -16048,8 +16374,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E74" s="14" t="n">
-        <v>7.8</v>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F74" s="12" t="n">
         <v>7</v>
@@ -16110,8 +16438,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E75" s="8" t="n">
-        <v>7.8</v>
+      <c r="E75" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F75" s="6" t="n">
         <v>1</v>
@@ -16173,7 +16503,7 @@
         </is>
       </c>
       <c r="E76" s="14" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F76" s="12" t="n">
         <v>5</v>
@@ -16235,7 +16565,7 @@
         </is>
       </c>
       <c r="E77" s="8" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="F77" s="6" t="n">
         <v>5</v>
@@ -16358,8 +16688,10 @@
           <t>Daniel Kwan &amp; Daniel Scheinert</t>
         </is>
       </c>
-      <c r="E79" s="8" t="n">
-        <v>7.8</v>
+      <c r="E79" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F79" s="6" t="n">
         <v>7</v>
@@ -16420,8 +16752,10 @@
           <t>Luc Besson</t>
         </is>
       </c>
-      <c r="E80" s="14" t="n">
-        <v>7.8</v>
+      <c r="E80" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F80" s="12" t="n">
         <v>0</v>
@@ -16482,8 +16816,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E81" s="8" t="n">
-        <v>7.8</v>
+      <c r="E81" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F81" s="6" t="n">
         <v>0</v>
@@ -16544,8 +16880,10 @@
           <t>Ridley Scott</t>
         </is>
       </c>
-      <c r="E82" s="14" t="n">
-        <v>7.8</v>
+      <c r="E82" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F82" s="12" t="n">
         <v>0</v>
@@ -16607,7 +16945,7 @@
         </is>
       </c>
       <c r="E83" s="8" t="n">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F83" s="6" t="n">
         <v>0</v>
@@ -16669,7 +17007,7 @@
         </is>
       </c>
       <c r="E84" s="14" t="n">
-        <v>7.7</v>
+        <v>6.8</v>
       </c>
       <c r="F84" s="12" t="n">
         <v>11</v>
@@ -16730,8 +17068,10 @@
           <t>Andrew Stanton</t>
         </is>
       </c>
-      <c r="E85" s="8" t="n">
-        <v>7.7</v>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F85" s="6" t="n">
         <v>1</v>
@@ -16792,8 +17132,10 @@
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="E86" s="14" t="n">
-        <v>7.7</v>
+      <c r="E86" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F86" s="12" t="n">
         <v>4</v>
@@ -16854,8 +17196,10 @@
           <t>Joel &amp; Ethan Coen</t>
         </is>
       </c>
-      <c r="E87" s="8" t="n">
-        <v>7.7</v>
+      <c r="E87" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F87" s="6" t="n">
         <v>4</v>
@@ -16916,8 +17260,10 @@
           <t>Brian De Palma</t>
         </is>
       </c>
-      <c r="E88" s="14" t="n">
-        <v>7.7</v>
+      <c r="E88" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F88" s="12" t="n">
         <v>0</v>
@@ -16979,7 +17325,7 @@
         </is>
       </c>
       <c r="E89" s="8" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="F89" s="6" t="n">
         <v>0</v>
@@ -17040,8 +17386,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E90" s="14" t="n">
-        <v>7.6</v>
+      <c r="E90" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F90" s="12" t="n">
         <v>4</v>
@@ -17102,8 +17450,10 @@
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="E91" s="8" t="n">
-        <v>7.6</v>
+      <c r="E91" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F91" s="6" t="n">
         <v>3</v>
@@ -17164,8 +17514,10 @@
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="E92" s="14" t="n">
-        <v>7.6</v>
+      <c r="E92" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F92" s="12" t="n">
         <v>2</v>
@@ -17227,7 +17579,7 @@
         </is>
       </c>
       <c r="E93" s="8" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="F93" s="6" t="n">
         <v>1</v>
@@ -17288,8 +17640,10 @@
           <t>Mel Gibson</t>
         </is>
       </c>
-      <c r="E94" s="14" t="n">
-        <v>7.6</v>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F94" s="12" t="n">
         <v>5</v>
@@ -17350,8 +17704,10 @@
           <t>Steve McQueen</t>
         </is>
       </c>
-      <c r="E95" s="8" t="n">
-        <v>7.6</v>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F95" s="6" t="n">
         <v>3</v>
@@ -17412,8 +17768,10 @@
           <t>Wes Anderson</t>
         </is>
       </c>
-      <c r="E96" s="14" t="n">
-        <v>7.6</v>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F96" s="12" t="n">
         <v>4</v>
@@ -17474,8 +17832,10 @@
           <t>Paul Thomas Anderson</t>
         </is>
       </c>
-      <c r="E97" s="8" t="n">
-        <v>7.6</v>
+      <c r="E97" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F97" s="6" t="n">
         <v>2</v>
@@ -17536,8 +17896,10 @@
           <t>Stanley Kubrick</t>
         </is>
       </c>
-      <c r="E98" s="14" t="n">
-        <v>7.6</v>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F98" s="12" t="n">
         <v>0</v>
@@ -17660,8 +18022,10 @@
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="E100" s="14" t="n">
-        <v>7.5</v>
+      <c r="E100" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F100" s="12" t="n">
         <v>0</v>
@@ -17722,8 +18086,10 @@
           <t>Todd Phillips</t>
         </is>
       </c>
-      <c r="E101" s="8" t="n">
-        <v>7.5</v>
+      <c r="E101" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F101" s="6" t="n">
         <v>2</v>
@@ -17784,8 +18150,10 @@
           <t>David Fincher</t>
         </is>
       </c>
-      <c r="E102" s="14" t="n">
-        <v>7.5</v>
+      <c r="E102" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F102" s="12" t="n">
         <v>3</v>
@@ -17847,7 +18215,7 @@
         </is>
       </c>
       <c r="E103" s="8" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="F103" s="6" t="n">
         <v>3</v>
@@ -17908,8 +18276,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E104" s="14" t="n">
-        <v>7.4</v>
+      <c r="E104" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F104" s="12" t="n">
         <v>0</v>
@@ -17970,8 +18340,10 @@
           <t>Byron Howard &amp; Rich Moore</t>
         </is>
       </c>
-      <c r="E105" s="8" t="n">
-        <v>7.4</v>
+      <c r="E105" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F105" s="6" t="n">
         <v>1</v>
@@ -18033,7 +18405,7 @@
         </is>
       </c>
       <c r="E106" s="14" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="F106" s="12" t="n">
         <v>0</v>
@@ -18094,8 +18466,10 @@
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="E107" s="8" t="n">
-        <v>7.3</v>
+      <c r="E107" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F107" s="6" t="n">
         <v>0</v>
@@ -18156,8 +18530,10 @@
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="E108" s="14" t="n">
-        <v>7.3</v>
+      <c r="E108" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F108" s="12" t="n">
         <v>4</v>
@@ -18218,8 +18594,10 @@
           <t>Barry Jenkins</t>
         </is>
       </c>
-      <c r="E109" s="8" t="n">
-        <v>7.3</v>
+      <c r="E109" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F109" s="6" t="n">
         <v>3</v>
@@ -18281,7 +18659,7 @@
         </is>
       </c>
       <c r="E110" s="14" t="n">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="F110" s="12" t="n">
         <v>0</v>
@@ -18342,8 +18720,10 @@
           <t>Joseph Kosinski</t>
         </is>
       </c>
-      <c r="E111" s="8" t="n">
-        <v>7.2</v>
+      <c r="E111" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F111" s="6" t="n">
         <v>1</v>
@@ -18404,8 +18784,10 @@
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="E112" s="14" t="n">
-        <v>7.2</v>
+      <c r="E112" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F112" s="12" t="n">
         <v>2</v>
@@ -18466,8 +18848,10 @@
           <t>Damien Chazelle</t>
         </is>
       </c>
-      <c r="E113" s="8" t="n">
-        <v>7.2</v>
+      <c r="E113" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F113" s="6" t="n">
         <v>6</v>
@@ -18528,8 +18912,10 @@
           <t>Chloé Zhao</t>
         </is>
       </c>
-      <c r="E114" s="14" t="n">
-        <v>7.2</v>
+      <c r="E114" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F114" s="12" t="n">
         <v>3</v>
@@ -18590,8 +18976,10 @@
           <t>Josh Cooley</t>
         </is>
       </c>
-      <c r="E115" s="8" t="n">
-        <v>7.1</v>
+      <c r="E115" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F115" s="6" t="n">
         <v>1</v>
@@ -18652,8 +19040,10 @@
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="E116" s="14" t="n">
-        <v>7.1</v>
+      <c r="E116" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F116" s="12" t="n">
         <v>0</v>
@@ -18714,8 +19104,10 @@
           <t>Francis Ford Coppola</t>
         </is>
       </c>
-      <c r="E117" s="8" t="n">
-        <v>7.1</v>
+      <c r="E117" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F117" s="6" t="n">
         <v>0</v>
@@ -18776,8 +19168,10 @@
           <t>Kelsey Mann</t>
         </is>
       </c>
-      <c r="E118" s="14" t="n">
-        <v>7</v>
+      <c r="E118" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F118" s="12" t="n">
         <v>1</v>
@@ -18838,8 +19232,10 @@
           <t>Shawn Levy</t>
         </is>
       </c>
-      <c r="E119" s="8" t="n">
-        <v>7</v>
+      <c r="E119" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F119" s="6" t="n">
         <v>0</v>
@@ -18901,7 +19297,7 @@
         </is>
       </c>
       <c r="E120" s="14" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="F120" s="12" t="n">
         <v>0</v>
@@ -18962,8 +19358,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E121" s="8" t="n">
-        <v>7</v>
+      <c r="E121" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F121" s="6" t="n">
         <v>0</v>
@@ -19024,8 +19422,10 @@
           <t>Mike Newell</t>
         </is>
       </c>
-      <c r="E122" s="14" t="n">
-        <v>7</v>
+      <c r="E122" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F122" s="12" t="n">
         <v>0</v>
@@ -19086,8 +19486,10 @@
           <t>Alfonso Cuarón</t>
         </is>
       </c>
-      <c r="E123" s="8" t="n">
-        <v>7</v>
+      <c r="E123" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F123" s="6" t="n">
         <v>7</v>
@@ -19148,8 +19550,10 @@
           <t>Guillermo del Toro</t>
         </is>
       </c>
-      <c r="E124" s="14" t="n">
-        <v>7</v>
+      <c r="E124" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F124" s="12" t="n">
         <v>4</v>
@@ -19211,7 +19615,7 @@
         </is>
       </c>
       <c r="E125" s="8" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="F125" s="6" t="n">
         <v>0</v>
@@ -19272,8 +19676,10 @@
           <t>Alejandro G. Iñárritu</t>
         </is>
       </c>
-      <c r="E126" s="14" t="n">
-        <v>6.9</v>
+      <c r="E126" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F126" s="12" t="n">
         <v>3</v>
@@ -19334,8 +19740,10 @@
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="E127" s="8" t="n">
-        <v>6.8</v>
+      <c r="E127" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F127" s="6" t="n">
         <v>0</v>
@@ -19397,7 +19805,7 @@
         </is>
       </c>
       <c r="E128" s="14" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="F128" s="12" t="n">
         <v>3</v>
@@ -19458,8 +19866,10 @@
           <t>Brad Bird</t>
         </is>
       </c>
-      <c r="E129" s="8" t="n">
-        <v>6.8</v>
+      <c r="E129" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F129" s="6" t="n">
         <v>0</v>
@@ -19520,8 +19930,10 @@
           <t>Gareth Edwards</t>
         </is>
       </c>
-      <c r="E130" s="14" t="n">
-        <v>6.8</v>
+      <c r="E130" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F130" s="12" t="n">
         <v>0</v>
@@ -19582,8 +19994,10 @@
           <t>Jon Favreau</t>
         </is>
       </c>
-      <c r="E131" s="8" t="n">
-        <v>6.8</v>
+      <c r="E131" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F131" s="6" t="n">
         <v>1</v>
@@ -19644,8 +20058,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E132" s="14" t="n">
-        <v>6.8</v>
+      <c r="E132" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F132" s="12" t="n">
         <v>0</v>
@@ -19706,8 +20122,10 @@
           <t>Andrew Adamson</t>
         </is>
       </c>
-      <c r="E133" s="8" t="n">
-        <v>6.8</v>
+      <c r="E133" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F133" s="6" t="n">
         <v>0</v>
@@ -19768,8 +20186,10 @@
           <t>David Yates</t>
         </is>
       </c>
-      <c r="E134" s="14" t="n">
-        <v>6.8</v>
+      <c r="E134" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F134" s="12" t="n">
         <v>0</v>
@@ -19830,8 +20250,10 @@
           <t>Chris Buck &amp; Jennifer Lee</t>
         </is>
       </c>
-      <c r="E135" s="8" t="n">
-        <v>6.7</v>
+      <c r="E135" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F135" s="6" t="n">
         <v>2</v>
@@ -19893,7 +20315,7 @@
         </is>
       </c>
       <c r="E136" s="14" t="n">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="F136" s="12" t="n">
         <v>0</v>
@@ -19954,8 +20376,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E137" s="8" t="n">
-        <v>6.7</v>
+      <c r="E137" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F137" s="6" t="n">
         <v>0</v>
@@ -20017,7 +20441,7 @@
         </is>
       </c>
       <c r="E138" s="14" t="n">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="F138" s="12" t="n">
         <v>0</v>
@@ -20078,8 +20502,10 @@
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="E139" s="8" t="n">
-        <v>6.7</v>
+      <c r="E139" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F139" s="6" t="n">
         <v>0</v>
@@ -20141,7 +20567,7 @@
         </is>
       </c>
       <c r="E140" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="F140" s="12" t="n">
         <v>1</v>
@@ -20202,8 +20628,10 @@
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="E141" s="8" t="n">
-        <v>6.6</v>
+      <c r="E141" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F141" s="6" t="n">
         <v>1</v>
@@ -20264,8 +20692,10 @@
           <t>Andrew Stanton</t>
         </is>
       </c>
-      <c r="E142" s="14" t="n">
-        <v>6.6</v>
+      <c r="E142" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F142" s="12" t="n">
         <v>0</v>
@@ -20326,8 +20756,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E143" s="8" t="n">
-        <v>6.6</v>
+      <c r="E143" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F143" s="6" t="n">
         <v>0</v>
@@ -20388,8 +20820,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E144" s="14" t="n">
-        <v>6.6</v>
+      <c r="E144" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F144" s="12" t="n">
         <v>0</v>
@@ -20450,8 +20884,10 @@
           <t>Greta Gerwig</t>
         </is>
       </c>
-      <c r="E145" s="8" t="n">
-        <v>6.5</v>
+      <c r="E145" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F145" s="6" t="n">
         <v>1</v>
@@ -20513,7 +20949,7 @@
         </is>
       </c>
       <c r="E146" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="F146" s="12" t="n">
         <v>0</v>
@@ -20574,8 +21010,10 @@
           <t>Bill Condon</t>
         </is>
       </c>
-      <c r="E147" s="8" t="n">
-        <v>6.4</v>
+      <c r="E147" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F147" s="6" t="n">
         <v>0</v>
@@ -20637,7 +21075,7 @@
         </is>
       </c>
       <c r="E148" s="14" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="F148" s="12" t="n">
         <v>0</v>
@@ -20698,8 +21136,10 @@
           <t>Jon Favreau</t>
         </is>
       </c>
-      <c r="E149" s="8" t="n">
-        <v>6.3</v>
+      <c r="E149" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F149" s="6" t="n">
         <v>0</v>
@@ -20760,8 +21200,10 @@
           <t>James Wan</t>
         </is>
       </c>
-      <c r="E150" s="14" t="n">
-        <v>6.2</v>
+      <c r="E150" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F150" s="12" t="n">
         <v>0</v>
@@ -20822,8 +21264,10 @@
           <t>Pierre Coffin &amp; Chris Renaud</t>
         </is>
       </c>
-      <c r="E151" s="8" t="n">
-        <v>6.2</v>
+      <c r="E151" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F151" s="6" t="n">
         <v>0</v>
@@ -20884,8 +21328,10 @@
           <t>Jake Kasdan</t>
         </is>
       </c>
-      <c r="E152" s="14" t="n">
-        <v>6.2</v>
+      <c r="E152" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F152" s="12" t="n">
         <v>0</v>
@@ -20946,8 +21392,10 @@
           <t>Guy Ritchie</t>
         </is>
       </c>
-      <c r="E153" s="8" t="n">
-        <v>6.1</v>
+      <c r="E153" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F153" s="6" t="n">
         <v>0</v>
@@ -21008,8 +21456,10 @@
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="E154" s="14" t="n">
-        <v>6.1</v>
+      <c r="E154" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F154" s="12" t="n">
         <v>0</v>
@@ -21070,8 +21520,10 @@
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="E155" s="8" t="n">
-        <v>6.1</v>
+      <c r="E155" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F155" s="6" t="n">
         <v>1</v>
@@ -21133,7 +21585,7 @@
         </is>
       </c>
       <c r="E156" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="F156" s="12" t="n">
         <v>0</v>
@@ -21194,8 +21646,10 @@
           <t>Aaron Horvath &amp; Michael Jelenic</t>
         </is>
       </c>
-      <c r="E157" s="8" t="n">
-        <v>6</v>
+      <c r="E157" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F157" s="6" t="n">
         <v>0</v>
@@ -21256,8 +21710,10 @@
           <t>Rian Johnson</t>
         </is>
       </c>
-      <c r="E158" s="14" t="n">
-        <v>6</v>
+      <c r="E158" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F158" s="12" t="n">
         <v>0</v>
@@ -21318,8 +21774,10 @@
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="E159" s="8" t="n">
-        <v>6</v>
+      <c r="E159" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F159" s="6" t="n">
         <v>0</v>
@@ -21381,7 +21839,7 @@
         </is>
       </c>
       <c r="E160" s="14" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="F160" s="12" t="n">
         <v>0</v>
@@ -21443,7 +21901,7 @@
         </is>
       </c>
       <c r="E161" s="8" t="n">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="F161" s="6" t="n">
         <v>1</v>
@@ -21504,8 +21962,10 @@
           <t>Chris Buck &amp; Jennifer Lee</t>
         </is>
       </c>
-      <c r="E162" s="14" t="n">
-        <v>5.9</v>
+      <c r="E162" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F162" s="12" t="n">
         <v>0</v>
@@ -21566,8 +22026,10 @@
           <t>James Wan</t>
         </is>
       </c>
-      <c r="E163" s="8" t="n">
-        <v>5.8</v>
+      <c r="E163" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F163" s="6" t="n">
         <v>0</v>
@@ -21628,8 +22090,10 @@
           <t>George Lucas</t>
         </is>
       </c>
-      <c r="E164" s="14" t="n">
-        <v>5.8</v>
+      <c r="E164" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F164" s="12" t="n">
         <v>0</v>
@@ -21690,8 +22154,10 @@
           <t>Tim Burton</t>
         </is>
       </c>
-      <c r="E165" s="8" t="n">
-        <v>5.8</v>
+      <c r="E165" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F165" s="6" t="n">
         <v>2</v>
@@ -21752,8 +22218,10 @@
           <t>Carlos Saldanha</t>
         </is>
       </c>
-      <c r="E166" s="14" t="n">
-        <v>5.8</v>
+      <c r="E166" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F166" s="12" t="n">
         <v>0</v>
@@ -21815,7 +22283,7 @@
         </is>
       </c>
       <c r="E167" s="8" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="F167" s="6" t="n">
         <v>0</v>
@@ -21876,8 +22344,10 @@
           <t>Kyle Balda</t>
         </is>
       </c>
-      <c r="E168" s="14" t="n">
-        <v>5.7</v>
+      <c r="E168" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F168" s="12" t="n">
         <v>0</v>
@@ -21938,8 +22408,10 @@
           <t>Chris Renaud</t>
         </is>
       </c>
-      <c r="E169" s="8" t="n">
-        <v>5.7</v>
+      <c r="E169" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F169" s="6" t="n">
         <v>0</v>
@@ -22000,8 +22472,10 @@
           <t>Chris Renaud</t>
         </is>
       </c>
-      <c r="E170" s="14" t="n">
-        <v>5.6</v>
+      <c r="E170" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F170" s="12" t="n">
         <v>0</v>
@@ -22124,8 +22598,10 @@
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="E172" s="14" t="n">
-        <v>5.5</v>
+      <c r="E172" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F172" s="12" t="n">
         <v>0</v>
@@ -22186,8 +22662,10 @@
           <t>David Derrick Jr.</t>
         </is>
       </c>
-      <c r="E173" s="8" t="n">
-        <v>5.5</v>
+      <c r="E173" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F173" s="6" t="n">
         <v>0</v>
@@ -22248,8 +22726,10 @@
           <t>Pierre Coffin &amp; Kyle Balda</t>
         </is>
       </c>
-      <c r="E174" s="14" t="n">
-        <v>5.5</v>
+      <c r="E174" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F174" s="12" t="n">
         <v>0</v>
@@ -22310,8 +22790,10 @@
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="E175" s="8" t="n">
-        <v>5.5</v>
+      <c r="E175" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F175" s="6" t="n">
         <v>0</v>
@@ -22372,8 +22854,10 @@
           <t>Zack Snyder</t>
         </is>
       </c>
-      <c r="E176" s="14" t="n">
-        <v>5.5</v>
+      <c r="E176" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F176" s="12" t="n">
         <v>0</v>
@@ -22434,8 +22918,10 @@
           <t>F. Gary Gray</t>
         </is>
       </c>
-      <c r="E177" s="8" t="n">
-        <v>5.4</v>
+      <c r="E177" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F177" s="6" t="n">
         <v>0</v>
@@ -22496,8 +22982,10 @@
           <t>Pierre Coffin &amp; Kyle Balda</t>
         </is>
       </c>
-      <c r="E178" s="14" t="n">
-        <v>5.4</v>
+      <c r="E178" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F178" s="12" t="n">
         <v>0</v>
@@ -22558,8 +23046,10 @@
           <t>Rob Marshall</t>
         </is>
       </c>
-      <c r="E179" s="8" t="n">
-        <v>5.4</v>
+      <c r="E179" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F179" s="6" t="n">
         <v>0</v>
@@ -22620,8 +23110,10 @@
           <t>Ruben Fleischer</t>
         </is>
       </c>
-      <c r="E180" s="14" t="n">
-        <v>5.4</v>
+      <c r="E180" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F180" s="12" t="n">
         <v>0</v>
@@ -22682,8 +23174,10 @@
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="E181" s="8" t="n">
-        <v>5.2</v>
+      <c r="E181" s="29" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F181" s="6" t="n">
         <v>0</v>
@@ -22744,8 +23238,10 @@
           <t>Steve Martino</t>
         </is>
       </c>
-      <c r="E182" s="14" t="n">
-        <v>5</v>
+      <c r="E182" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F182" s="12" t="n">
         <v>0</v>
@@ -22868,8 +23364,10 @@
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="E184" s="14" t="n">
-        <v>4.5</v>
+      <c r="E184" s="30" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="F184" s="12" t="n">
         <v>0</v>
@@ -23122,10 +23620,8 @@
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="E188" s="17" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
+      <c r="E188" s="14" t="n">
+        <v>6.3</v>
       </c>
       <c r="F188" s="12" t="n">
         <v>0</v>

</xml_diff>